<commit_message>
Update bom to indicate 10t pinion
Update bom to indicate 10t pinion for extruder stepper
</commit_message>
<xml_diff>
--- a/BOM/Lineux Hotswap BOM Beta.xlsx
+++ b/BOM/Lineux Hotswap BOM Beta.xlsx
@@ -28,108 +28,108 @@
     <t>Bom is for Ebb36 Toolboard. Other toolboard may need different hardwares.</t>
   </si>
   <si>
+    <t>Lineux Hotswap Voron Carriage</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
     <t>Lineux Hotswap Vzbot Carriage</t>
   </si>
   <si>
-    <t>Quantity</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
     <t>Source link</t>
   </si>
   <si>
     <t>Remarks</t>
   </si>
   <si>
+    <t>m3x5x4 brass insert</t>
+  </si>
+  <si>
+    <t>m3 hex nut</t>
+  </si>
+  <si>
     <t>Bom is based on V6 ChP. Other hotends may require different hardwares.</t>
   </si>
   <si>
-    <t>m3x5x4 brass insert</t>
+    <t>m3 x 6mm bhcs</t>
+  </si>
+  <si>
+    <t>m3 x 8mm set screw</t>
   </si>
   <si>
     <t>Lineux Hotswap Toolhead</t>
   </si>
   <si>
-    <t>Lineux Hotswap Voron Carriage</t>
-  </si>
-  <si>
-    <t>m3 hex nut</t>
+    <t>m3 x 6mm shcs</t>
   </si>
   <si>
     <t>m2.5 x 6mm shcs</t>
   </si>
   <si>
-    <t>m3 x 8mm set screw</t>
+    <t>m3 x 8mm shcs</t>
   </si>
   <si>
     <t>For V6 CHP</t>
   </si>
   <si>
-    <t>m3 x 6mm shcs</t>
-  </si>
-  <si>
     <t>Heatsink Mounting Screw</t>
   </si>
   <si>
-    <t>m3 x 8mm shcs</t>
+    <t>m3 x 15mm shcs</t>
+  </si>
+  <si>
+    <t>m3 x 20mm shcs</t>
   </si>
   <si>
     <t>m3 x 10mm shcs</t>
   </si>
   <si>
+    <t>m3 x 25mm bhcs</t>
+  </si>
+  <si>
+    <t>m3 x 12mm shcs</t>
+  </si>
+  <si>
     <t>m3 x 16mm shcs</t>
   </si>
   <si>
-    <t>m3 x 20mm shcs</t>
-  </si>
-  <si>
-    <t>m3 x 6mm bhcs</t>
-  </si>
-  <si>
-    <t>m3 x 25mm bhcs</t>
+    <t>m3 x 30mm bhcs</t>
   </si>
   <si>
     <t>m3 x 6mm fhcs</t>
   </si>
   <si>
-    <t>m3 x 30mm bhcs</t>
-  </si>
-  <si>
-    <t>m3 x 12mm shcs</t>
-  </si>
-  <si>
     <t>m3 x 30mm shcs</t>
   </si>
   <si>
+    <t>m3 x 45mm shcs</t>
+  </si>
+  <si>
+    <t>m3 cap nut din1587</t>
+  </si>
+  <si>
+    <t>link</t>
+  </si>
+  <si>
     <t>m3 x 10mm bhcs</t>
   </si>
   <si>
+    <t>m3 x 20mm dowel pin</t>
+  </si>
+  <si>
     <t>m3 x 12mm bhcs</t>
   </si>
   <si>
-    <t>m3 x 45mm shcs</t>
-  </si>
-  <si>
     <t>m3 x 15mm bhcs</t>
   </si>
   <si>
     <t>m3 x 16mm also possible</t>
   </si>
   <si>
-    <t>m3 cap nut din1587</t>
-  </si>
-  <si>
-    <t>link</t>
-  </si>
-  <si>
-    <t>m3 x 15mm shcs</t>
-  </si>
-  <si>
-    <t>m3 x 20mm dowel pin</t>
-  </si>
-  <si>
     <t>m3 x 30mm dowel pin</t>
   </si>
   <si>
@@ -139,16 +139,58 @@
     <t>5x7x3</t>
   </si>
   <si>
+    <t>mr63zz bearing</t>
+  </si>
+  <si>
+    <t>U need 2 extra. Not from HGX Lite kit</t>
+  </si>
+  <si>
+    <t>8 x 5mm n52 magnet</t>
+  </si>
+  <si>
+    <t>microswitch</t>
+  </si>
+  <si>
+    <t>ws2812 Addressable Led</t>
+  </si>
+  <si>
+    <t>Nema 14 10t Stepper motor</t>
+  </si>
+  <si>
+    <t>HGX Lite Gears</t>
+  </si>
+  <si>
+    <t>Gear Kit</t>
+  </si>
+  <si>
+    <t>HGX Gears</t>
+  </si>
+  <si>
+    <t>Take note its not HGX Lite V2</t>
+  </si>
+  <si>
+    <t>Toolboard</t>
+  </si>
+  <si>
+    <t>Ebb36, H36, SHT36, Tool Lite, etc</t>
+  </si>
+  <si>
+    <t>5015 Radial Fan</t>
+  </si>
+  <si>
     <t>6 x 3mm n52 magnet</t>
   </si>
   <si>
-    <t>8 x 5mm n52 magnet</t>
+    <t>Ebb36, H36, SHT36 etc</t>
+  </si>
+  <si>
+    <t>Lineux Hotswap Voron Dock</t>
   </si>
   <si>
     <t>3010 Axial Fan</t>
   </si>
   <si>
-    <t>mr63zz bearing</t>
+    <t>Lineux Hotswap Vzbot Dock</t>
   </si>
   <si>
     <t>between 9-12mm width</t>
@@ -157,12 +199,12 @@
     <t>Length depends on printer size</t>
   </si>
   <si>
-    <t>U need 2 extra. Not from HGX Lite kit</t>
-  </si>
-  <si>
     <t>Industrial ziptie (between 9-10mm width recommended)</t>
   </si>
   <si>
+    <t>m3 washer</t>
+  </si>
+  <si>
     <t>For umbilical</t>
   </si>
   <si>
@@ -175,73 +217,34 @@
     <t>Can use Molex 2x3p as an alternative</t>
   </si>
   <si>
-    <t>microswitch</t>
-  </si>
-  <si>
-    <t>ws2812 Addressable Led</t>
-  </si>
-  <si>
-    <t>Nema 14 Stepper motor</t>
-  </si>
-  <si>
-    <t>HGX Lite Gears</t>
-  </si>
-  <si>
-    <t>Gear Kit</t>
-  </si>
-  <si>
-    <t>HGX Gears</t>
-  </si>
-  <si>
-    <t>Take note its not HGX Lite V2</t>
-  </si>
-  <si>
-    <t>Toolboard</t>
-  </si>
-  <si>
-    <t>Ebb36, H36, SHT36, Tool Lite, etc</t>
-  </si>
-  <si>
-    <t>5015 Radial Fan</t>
-  </si>
-  <si>
-    <t>Ebb36, H36, SHT36 etc</t>
+    <t>m3 od5 35mm threaded dowel pin</t>
+  </si>
+  <si>
+    <t>5x35xM3</t>
+  </si>
+  <si>
+    <t>Silicon Brush</t>
+  </si>
+  <si>
+    <t>Can be cut into 2 or 3 per piece</t>
+  </si>
+  <si>
+    <t>AA battery terminal</t>
   </si>
   <si>
     <t>Lineux Hotswap Voron CNC Tap Dock</t>
   </si>
   <si>
-    <t>Lineux Hotswap Vzbot Dock</t>
-  </si>
-  <si>
     <t>Take note of the type</t>
   </si>
   <si>
-    <t>m3 washer</t>
-  </si>
-  <si>
     <t>jst xh 4pin male</t>
   </si>
   <si>
     <t>molex 1x2pin male</t>
   </si>
   <si>
-    <t>m3 od5 35mm threaded dowel pin</t>
-  </si>
-  <si>
-    <t>5x35xM3</t>
-  </si>
-  <si>
-    <t>Silicon Brush</t>
-  </si>
-  <si>
-    <t>Lineux Hotswap Voron Dock</t>
-  </si>
-  <si>
-    <t>Can be cut into 2 or 3 per piece</t>
-  </si>
-  <si>
-    <t>AA battery terminal</t>
+    <t>Take note of dimension</t>
   </si>
   <si>
     <t>Take note of the clip position</t>
@@ -263,9 +266,6 @@
   </si>
   <si>
     <t>Depends on your choice</t>
-  </si>
-  <si>
-    <t>Take note of dimension</t>
   </si>
 </sst>
 </file>
@@ -500,21 +500,21 @@
     <xf borderId="11" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
+    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="6" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="6" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
     <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -522,23 +522,23 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="5" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="6" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" vertical="bottom"/>
+    </xf>
     <xf borderId="5" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="6" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -806,7 +806,7 @@
     </row>
     <row r="6">
       <c r="A6" s="8" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>5</v>
@@ -815,10 +815,10 @@
         <v>6</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -834,7 +834,7 @@
     </row>
     <row r="8">
       <c r="A8" s="16" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B8" s="13">
         <v>1.0</v>
@@ -845,7 +845,7 @@
     </row>
     <row r="9">
       <c r="A9" s="16" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="B9" s="13">
         <v>3.0</v>
@@ -856,7 +856,7 @@
     </row>
     <row r="10">
       <c r="A10" s="16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B10" s="13">
         <v>1.0</v>
@@ -867,7 +867,7 @@
     </row>
     <row r="11">
       <c r="A11" s="18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B11" s="19">
         <v>3.0</v>
@@ -878,7 +878,7 @@
     </row>
     <row r="12">
       <c r="A12" s="16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B12" s="13">
         <v>5.0</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="13">
       <c r="A13" s="16" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="B13" s="13">
         <v>4.0</v>
@@ -922,7 +922,7 @@
     </row>
     <row r="16">
       <c r="A16" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B16" s="13">
         <v>4.0</v>
@@ -933,7 +933,7 @@
     </row>
     <row r="17">
       <c r="A17" s="16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B17" s="13">
         <v>1.0</v>
@@ -944,7 +944,7 @@
     </row>
     <row r="18">
       <c r="A18" s="16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B18" s="13">
         <v>2.0</v>
@@ -955,19 +955,19 @@
     </row>
     <row r="19">
       <c r="A19" s="18" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B19" s="19">
         <v>3.0</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E19" s="15"/>
     </row>
     <row r="20">
       <c r="A20" s="16" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B20" s="13">
         <v>2.0</v>
@@ -998,13 +998,13 @@
         <v>40</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E22" s="15"/>
     </row>
     <row r="23">
       <c r="A23" s="16" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B23" s="13">
         <v>2.0</v>
@@ -1012,12 +1012,12 @@
       <c r="C23" s="14"/>
       <c r="D23" s="14"/>
       <c r="E23" s="25" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B24" s="13">
         <v>3.0</v>
@@ -1028,7 +1028,7 @@
     </row>
     <row r="25">
       <c r="A25" s="16" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="B25" s="13">
         <v>1.0</v>
@@ -1039,7 +1039,7 @@
     </row>
     <row r="26">
       <c r="A26" s="12" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="B26" s="13">
         <v>2.0</v>
@@ -1050,7 +1050,7 @@
     </row>
     <row r="27">
       <c r="A27" s="16" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="B27" s="13">
         <v>1.0</v>
@@ -1061,24 +1061,24 @@
     </row>
     <row r="28">
       <c r="A28" s="16" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="B28" s="13">
         <v>1.0</v>
       </c>
       <c r="C28" s="24" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E28" s="25" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="16" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B29" s="13">
         <v>1.0</v>
@@ -1086,23 +1086,23 @@
       <c r="C29" s="14"/>
       <c r="D29" s="14"/>
       <c r="E29" s="25" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="27" t="s">
-        <v>62</v>
-      </c>
-      <c r="B30" s="28">
-        <v>1.0</v>
-      </c>
-      <c r="C30" s="29"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="30"/>
+      <c r="A30" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="B30" s="27">
+        <v>1.0</v>
+      </c>
+      <c r="C30" s="28"/>
+      <c r="D30" s="28"/>
+      <c r="E30" s="29"/>
     </row>
     <row r="32">
       <c r="A32" s="8" t="s">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="B32" s="9" t="s">
         <v>5</v>
@@ -1111,10 +1111,10 @@
         <v>6</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="33">
@@ -1128,7 +1128,7 @@
     </row>
     <row r="34">
       <c r="A34" s="18" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B34" s="19">
         <v>1.0</v>
@@ -1137,7 +1137,7 @@
     </row>
     <row r="35">
       <c r="A35" s="18" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B35" s="19">
         <v>2.0</v>
@@ -1146,7 +1146,7 @@
     </row>
     <row r="36">
       <c r="A36" s="18" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B36" s="19">
         <v>3.0</v>
@@ -1155,7 +1155,7 @@
     </row>
     <row r="37">
       <c r="A37" s="18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B37" s="19">
         <v>3.0</v>
@@ -1164,7 +1164,7 @@
     </row>
     <row r="38">
       <c r="A38" s="18" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B38" s="19">
         <v>4.0</v>
@@ -1173,22 +1173,22 @@
     </row>
     <row r="39">
       <c r="A39" s="18" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B39" s="19">
         <v>1.0</v>
       </c>
       <c r="C39" s="19" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E39" s="21"/>
     </row>
     <row r="40">
       <c r="A40" s="12" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="B40" s="19">
         <v>1.0</v>
@@ -1197,36 +1197,36 @@
     </row>
     <row r="41">
       <c r="A41" s="16" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B41" s="19">
         <v>1.0</v>
       </c>
       <c r="D41" s="23" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E41" s="20" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="31" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B42" s="32">
         <v>1.0</v>
       </c>
       <c r="C42" s="33"/>
-      <c r="D42" s="36" t="s">
-        <v>35</v>
+      <c r="D42" s="34" t="s">
+        <v>32</v>
       </c>
       <c r="E42" s="35" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="37"/>
-      <c r="B43" s="38"/>
+      <c r="A43" s="36"/>
+      <c r="B43" s="37"/>
       <c r="C43" s="14"/>
       <c r="D43" s="14"/>
       <c r="E43" s="14"/>
@@ -1303,7 +1303,7 @@
     </row>
     <row r="54">
       <c r="A54" s="24"/>
-      <c r="B54" s="39"/>
+      <c r="B54" s="38"/>
       <c r="C54" s="24"/>
       <c r="D54" s="22"/>
       <c r="E54" s="14"/>
@@ -1345,7 +1345,7 @@
     </row>
     <row r="60">
       <c r="A60" s="14"/>
-      <c r="B60" s="39"/>
+      <c r="B60" s="38"/>
       <c r="C60" s="14"/>
       <c r="D60" s="14"/>
       <c r="E60" s="14"/>
@@ -1375,8 +1375,8 @@
       <c r="A64" s="19"/>
     </row>
     <row r="69">
-      <c r="A69" s="37"/>
-      <c r="B69" s="38"/>
+      <c r="A69" s="36"/>
+      <c r="B69" s="37"/>
       <c r="C69" s="14"/>
       <c r="D69" s="14"/>
       <c r="E69" s="14"/>
@@ -1446,8 +1446,8 @@
       <c r="D86" s="22"/>
     </row>
     <row r="88">
-      <c r="A88" s="37"/>
-      <c r="B88" s="38"/>
+      <c r="A88" s="36"/>
+      <c r="B88" s="37"/>
       <c r="C88" s="14"/>
       <c r="D88" s="14"/>
       <c r="E88" s="14"/>
@@ -1557,7 +1557,7 @@
     </row>
     <row r="6">
       <c r="A6" s="8" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>5</v>
@@ -1566,10 +1566,10 @@
         <v>6</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -1585,7 +1585,7 @@
     </row>
     <row r="8">
       <c r="A8" s="16" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B8" s="13">
         <v>1.0</v>
@@ -1596,7 +1596,7 @@
     </row>
     <row r="9">
       <c r="A9" s="16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B9" s="13">
         <v>6.0</v>
@@ -1607,7 +1607,7 @@
     </row>
     <row r="10">
       <c r="A10" s="18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B10" s="19">
         <v>3.0</v>
@@ -1618,7 +1618,7 @@
     </row>
     <row r="11">
       <c r="A11" s="16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B11" s="13">
         <v>7.0</v>
@@ -1629,7 +1629,7 @@
     </row>
     <row r="12">
       <c r="A12" s="16" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B12" s="13">
         <v>2.0</v>
@@ -1662,7 +1662,7 @@
     </row>
     <row r="15">
       <c r="A15" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B15" s="13">
         <v>4.0</v>
@@ -1673,7 +1673,7 @@
     </row>
     <row r="16">
       <c r="A16" s="16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B16" s="13">
         <v>1.0</v>
@@ -1684,7 +1684,7 @@
     </row>
     <row r="17">
       <c r="A17" s="16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B17" s="13">
         <v>2.0</v>
@@ -1695,7 +1695,7 @@
     </row>
     <row r="18">
       <c r="A18" s="18" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B18" s="19">
         <v>2.0</v>
@@ -1715,13 +1715,13 @@
     </row>
     <row r="20">
       <c r="A20" s="18" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B20" s="19">
         <v>3.0</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E20" s="15"/>
     </row>
@@ -1736,13 +1736,13 @@
         <v>40</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E21" s="15"/>
     </row>
     <row r="22">
       <c r="A22" s="16" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B22" s="13">
         <v>2.0</v>
@@ -1750,12 +1750,12 @@
       <c r="C22" s="14"/>
       <c r="D22" s="14"/>
       <c r="E22" s="25" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B23" s="13">
         <v>3.0</v>
@@ -1766,7 +1766,7 @@
     </row>
     <row r="24">
       <c r="A24" s="16" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="B24" s="13">
         <v>1.0</v>
@@ -1777,7 +1777,7 @@
     </row>
     <row r="25">
       <c r="A25" s="12" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="B25" s="13">
         <v>2.0</v>
@@ -1788,7 +1788,7 @@
     </row>
     <row r="26">
       <c r="A26" s="16" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="B26" s="13">
         <v>1.0</v>
@@ -1799,24 +1799,24 @@
     </row>
     <row r="27">
       <c r="A27" s="16" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="B27" s="13">
         <v>1.0</v>
       </c>
       <c r="C27" s="24" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E27" s="25" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="16" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B28" s="13">
         <v>1.0</v>
@@ -1824,23 +1824,23 @@
       <c r="C28" s="14"/>
       <c r="D28" s="14"/>
       <c r="E28" s="25" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="27" t="s">
-        <v>62</v>
-      </c>
-      <c r="B29" s="28">
-        <v>1.0</v>
-      </c>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="30"/>
+      <c r="A29" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="B29" s="27">
+        <v>1.0</v>
+      </c>
+      <c r="C29" s="28"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="29"/>
     </row>
     <row r="31">
       <c r="A31" s="8" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="B31" s="9" t="s">
         <v>5</v>
@@ -1849,10 +1849,10 @@
         <v>6</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="32">
@@ -1866,7 +1866,7 @@
     </row>
     <row r="33">
       <c r="A33" s="18" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B33" s="19">
         <v>1.0</v>
@@ -1875,7 +1875,7 @@
     </row>
     <row r="34">
       <c r="A34" s="18" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B34" s="19">
         <v>2.0</v>
@@ -1884,7 +1884,7 @@
     </row>
     <row r="35">
       <c r="A35" s="18" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B35" s="19">
         <v>3.0</v>
@@ -1893,7 +1893,7 @@
     </row>
     <row r="36">
       <c r="A36" s="18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B36" s="19">
         <v>3.0</v>
@@ -1902,7 +1902,7 @@
     </row>
     <row r="37">
       <c r="A37" s="18" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B37" s="19">
         <v>4.0</v>
@@ -1911,22 +1911,22 @@
     </row>
     <row r="38">
       <c r="A38" s="18" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B38" s="19">
         <v>1.0</v>
       </c>
       <c r="C38" s="19" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D38" s="23" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E38" s="21"/>
     </row>
     <row r="39">
       <c r="A39" s="12" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="B39" s="19">
         <v>1.0</v>
@@ -1935,36 +1935,36 @@
     </row>
     <row r="40">
       <c r="A40" s="16" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B40" s="19">
         <v>1.0</v>
       </c>
       <c r="D40" s="23" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E40" s="20" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="31" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B41" s="32">
         <v>1.0</v>
       </c>
       <c r="C41" s="33"/>
-      <c r="D41" s="36" t="s">
-        <v>35</v>
+      <c r="D41" s="34" t="s">
+        <v>32</v>
       </c>
       <c r="E41" s="35" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="37"/>
-      <c r="B42" s="38"/>
+      <c r="A42" s="36"/>
+      <c r="B42" s="37"/>
       <c r="C42" s="14"/>
       <c r="D42" s="14"/>
       <c r="E42" s="14"/>
@@ -2041,7 +2041,7 @@
     </row>
     <row r="53">
       <c r="A53" s="24"/>
-      <c r="B53" s="39"/>
+      <c r="B53" s="38"/>
       <c r="C53" s="24"/>
       <c r="D53" s="22"/>
       <c r="E53" s="14"/>
@@ -2083,7 +2083,7 @@
     </row>
     <row r="59">
       <c r="A59" s="14"/>
-      <c r="B59" s="39"/>
+      <c r="B59" s="38"/>
       <c r="C59" s="14"/>
       <c r="D59" s="14"/>
       <c r="E59" s="14"/>
@@ -2113,8 +2113,8 @@
       <c r="A63" s="19"/>
     </row>
     <row r="68">
-      <c r="A68" s="37"/>
-      <c r="B68" s="38"/>
+      <c r="A68" s="36"/>
+      <c r="B68" s="37"/>
       <c r="C68" s="14"/>
       <c r="D68" s="14"/>
       <c r="E68" s="14"/>
@@ -2184,8 +2184,8 @@
       <c r="D85" s="22"/>
     </row>
     <row r="87">
-      <c r="A87" s="37"/>
-      <c r="B87" s="38"/>
+      <c r="A87" s="36"/>
+      <c r="B87" s="37"/>
       <c r="C87" s="14"/>
       <c r="D87" s="14"/>
       <c r="E87" s="14"/>
@@ -2295,7 +2295,7 @@
     </row>
     <row r="6">
       <c r="A6" s="8" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>5</v>
@@ -2304,10 +2304,10 @@
         <v>6</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -2323,7 +2323,7 @@
     </row>
     <row r="8">
       <c r="A8" s="16" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B8" s="13">
         <v>3.0</v>
@@ -2334,7 +2334,7 @@
     </row>
     <row r="9">
       <c r="A9" s="18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B9" s="19">
         <v>3.0</v>
@@ -2345,7 +2345,7 @@
     </row>
     <row r="10">
       <c r="A10" s="16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B10" s="13">
         <v>14.0</v>
@@ -2356,7 +2356,7 @@
     </row>
     <row r="11">
       <c r="A11" s="16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B11" s="13">
         <v>7.0</v>
@@ -2367,7 +2367,7 @@
     </row>
     <row r="12">
       <c r="A12" s="16" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B12" s="13">
         <v>2.0</v>
@@ -2378,7 +2378,7 @@
     </row>
     <row r="13">
       <c r="A13" s="16" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B13" s="13">
         <v>2.0</v>
@@ -2411,7 +2411,7 @@
     </row>
     <row r="16">
       <c r="A16" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B16" s="13">
         <v>4.0</v>
@@ -2422,7 +2422,7 @@
     </row>
     <row r="17">
       <c r="A17" s="16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B17" s="13">
         <v>1.0</v>
@@ -2433,7 +2433,7 @@
     </row>
     <row r="18">
       <c r="A18" s="16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B18" s="13">
         <v>2.0</v>
@@ -2444,13 +2444,13 @@
     </row>
     <row r="19">
       <c r="A19" s="18" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B19" s="19">
         <v>3.0</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E19" s="15"/>
     </row>
@@ -2465,13 +2465,13 @@
         <v>40</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E20" s="15"/>
     </row>
     <row r="21">
       <c r="A21" s="16" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B21" s="13">
         <v>4.0</v>
@@ -2493,7 +2493,7 @@
     </row>
     <row r="23">
       <c r="A23" s="16" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B23" s="13">
         <v>2.0</v>
@@ -2501,12 +2501,12 @@
       <c r="C23" s="14"/>
       <c r="D23" s="14"/>
       <c r="E23" s="25" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B24" s="13">
         <v>3.0</v>
@@ -2517,7 +2517,7 @@
     </row>
     <row r="25">
       <c r="A25" s="16" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="B25" s="13">
         <v>1.0</v>
@@ -2528,7 +2528,7 @@
     </row>
     <row r="26">
       <c r="A26" s="12" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="B26" s="13">
         <v>3.0</v>
@@ -2539,7 +2539,7 @@
     </row>
     <row r="27">
       <c r="A27" s="16" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="B27" s="13">
         <v>1.0</v>
@@ -2550,24 +2550,24 @@
     </row>
     <row r="28">
       <c r="A28" s="16" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="B28" s="13">
         <v>1.0</v>
       </c>
       <c r="C28" s="24" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E28" s="25" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="16" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B29" s="13">
         <v>1.0</v>
@@ -2575,23 +2575,23 @@
       <c r="C29" s="14"/>
       <c r="D29" s="14"/>
       <c r="E29" s="25" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="27" t="s">
-        <v>62</v>
-      </c>
-      <c r="B30" s="28">
-        <v>1.0</v>
-      </c>
-      <c r="C30" s="29"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="30"/>
+      <c r="A30" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="B30" s="27">
+        <v>1.0</v>
+      </c>
+      <c r="C30" s="28"/>
+      <c r="D30" s="28"/>
+      <c r="E30" s="29"/>
     </row>
     <row r="32">
       <c r="A32" s="8" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="B32" s="9" t="s">
         <v>5</v>
@@ -2600,10 +2600,10 @@
         <v>6</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="33">
@@ -2617,7 +2617,7 @@
     </row>
     <row r="34">
       <c r="A34" s="18" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B34" s="19">
         <v>1.0</v>
@@ -2626,7 +2626,7 @@
     </row>
     <row r="35">
       <c r="A35" s="18" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B35" s="19">
         <v>2.0</v>
@@ -2635,7 +2635,7 @@
     </row>
     <row r="36">
       <c r="A36" s="18" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B36" s="19">
         <v>3.0</v>
@@ -2644,7 +2644,7 @@
     </row>
     <row r="37">
       <c r="A37" s="18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B37" s="19">
         <v>5.0</v>
@@ -2653,7 +2653,7 @@
     </row>
     <row r="38">
       <c r="A38" s="18" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B38" s="19">
         <v>2.0</v>
@@ -2662,22 +2662,22 @@
     </row>
     <row r="39">
       <c r="A39" s="18" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B39" s="19">
         <v>1.0</v>
       </c>
       <c r="C39" s="19" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E39" s="21"/>
     </row>
     <row r="40">
       <c r="A40" s="12" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="B40" s="19">
         <v>1.0</v>
@@ -2686,31 +2686,31 @@
     </row>
     <row r="41">
       <c r="A41" s="16" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B41" s="19">
         <v>1.0</v>
       </c>
       <c r="D41" s="23" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E41" s="20" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="31" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B42" s="32">
         <v>1.0</v>
       </c>
       <c r="C42" s="33"/>
-      <c r="D42" s="36" t="s">
-        <v>35</v>
+      <c r="D42" s="34" t="s">
+        <v>32</v>
       </c>
       <c r="E42" s="35" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -2766,12 +2766,12 @@
     </row>
     <row r="3">
       <c r="A3" s="7" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B5" s="9" t="s">
         <v>5</v>
@@ -2780,24 +2780,24 @@
         <v>6</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="18" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B6" s="19">
         <v>4.0</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7">
@@ -2811,7 +2811,7 @@
     </row>
     <row r="8">
       <c r="A8" s="18" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B8" s="19">
         <v>1.0</v>
@@ -2820,7 +2820,7 @@
     </row>
     <row r="9">
       <c r="A9" s="18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B9" s="19">
         <v>1.0</v>
@@ -2829,7 +2829,7 @@
     </row>
     <row r="10">
       <c r="A10" s="18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B10" s="19">
         <v>2.0</v>
@@ -2838,7 +2838,7 @@
     </row>
     <row r="11">
       <c r="A11" s="18" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B11" s="19">
         <v>2.0</v>
@@ -2847,7 +2847,7 @@
     </row>
     <row r="12">
       <c r="A12" s="18" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B12" s="19">
         <v>2.0</v>
@@ -2856,24 +2856,24 @@
     </row>
     <row r="13">
       <c r="A13" s="18" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B13" s="19">
         <v>2.0</v>
       </c>
       <c r="E13" s="20" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="18" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B14" s="19">
         <v>1.0</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E14" s="21"/>
     </row>
@@ -2888,13 +2888,13 @@
         <v>40</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E15" s="21"/>
     </row>
     <row r="16">
       <c r="A16" s="12" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="B16" s="13">
         <v>1.0</v>
@@ -2903,7 +2903,7 @@
     </row>
     <row r="17">
       <c r="A17" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B17" s="13">
         <v>3.0</v>
@@ -2912,53 +2912,53 @@
     </row>
     <row r="18">
       <c r="A18" s="18" t="s">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="B18" s="19">
         <v>1.0</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="D18" s="22"/>
       <c r="E18" s="20" t="s">
-        <v>46</v>
+        <v>60</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="18" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="B19" s="19">
         <v>1.0</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="E19" s="20" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="18" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
       <c r="B20" s="19">
         <v>1.0</v>
       </c>
-      <c r="C20" s="26" t="s">
-        <v>52</v>
+      <c r="C20" s="30" t="s">
+        <v>66</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E20" s="20" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="18" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="B21" s="19">
         <v>1.0</v>
@@ -2968,54 +2968,54 @@
     </row>
     <row r="22">
       <c r="A22" s="18" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="B22" s="19">
         <v>1.0</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E22" s="20" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B23" s="19">
         <v>1.0</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E23" s="21"/>
     </row>
     <row r="24">
       <c r="A24" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B24" s="19">
         <v>1.0</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D24" s="22"/>
       <c r="E24" s="20" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="31" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B25" s="32"/>
       <c r="C25" s="33"/>
-      <c r="D25" s="34"/>
+      <c r="D25" s="39"/>
       <c r="E25" s="35" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>